<commit_message>
Kontaktimport: Firma und Mitarbeiternummer fuer Mitarbeiter automatisch setzen.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/testdata/import-fixtures/kontakte/kontakte-excel.xlsx
+++ b/docs/testdata/import-fixtures/kontakte/kontakte-excel.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>Anrede</t>
   </si>
@@ -19,6 +19,9 @@
     <t>Nachname</t>
   </si>
   <si>
+    <t>Firma</t>
+  </si>
+  <si>
     <t>E-Mail</t>
   </si>
   <si>
@@ -28,10 +31,13 @@
     <t>Login</t>
   </si>
   <si>
+    <t>Kundennummer</t>
+  </si>
+  <si>
     <t>Rolle</t>
   </si>
   <si>
-    <t>Frau/Herr</t>
+    <t>Frau</t>
   </si>
   <si>
     <t>Anna</t>
@@ -40,6 +46,9 @@
     <t>Duplikat</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>anna.duplikat@demo-import.ganz-om.invalid</t>
   </si>
   <si>
@@ -50,6 +59,9 @@
   </si>
   <si>
     <t>mitarbeiter</t>
+  </si>
+  <si>
+    <t>Herr</t>
   </si>
   <si>
     <t>Bernd</t>
@@ -244,281 +256,359 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>32</v>
+      </c>
+      <c r="H5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>37</v>
+      </c>
+      <c r="H6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>47</v>
+      </c>
+      <c r="H8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>52</v>
+      </c>
+      <c r="H9" t="s">
+        <v>12</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F10" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G10" t="s">
-        <v>13</v>
+        <v>57</v>
+      </c>
+      <c r="H10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>62</v>
+      </c>
+      <c r="H11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F12" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G12" t="s">
-        <v>13</v>
+        <v>67</v>
+      </c>
+      <c r="H12" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F13" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G13" t="s">
-        <v>13</v>
+        <v>72</v>
+      </c>
+      <c r="H13" t="s">
+        <v>12</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>